<commit_message>
Introducir fortuna para tester y cambiar ciclismo con gimnasia
</commit_message>
<xml_diff>
--- a/datos/deportes.xlsx
+++ b/datos/deportes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manue\OneDrive\Desktop\Juegos\Road to Gold\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A4FB406-45CE-404B-BDBA-3536740808B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DFF6203-0380-4830-905D-12E053BAABDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0C12F03E-F4F1-4B58-AEF9-00A818977629}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="61">
   <si>
     <t>id</t>
   </si>
@@ -219,6 +219,9 @@
   </si>
   <si>
     <t>aventura</t>
+  </si>
+  <si>
+    <t>fijo_alternativo</t>
   </si>
 </sst>
 </file>
@@ -712,10 +715,10 @@
         <v>18</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="E4">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F4">
         <v>3</v>
@@ -852,16 +855,16 @@
         <v>27</v>
       </c>
       <c r="D8" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="E8">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F8">
         <v>3</v>
       </c>
       <c r="G8">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="H8" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
meter rugby, tiro con arco y austria
</commit_message>
<xml_diff>
--- a/datos/deportes.xlsx
+++ b/datos/deportes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manue\OneDrive\Desktop\Juegos\Road to Gold\datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DFF6203-0380-4830-905D-12E053BAABDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFE686F0-2EA0-4B00-B08A-0EED5D1AFBCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0C12F03E-F4F1-4B58-AEF9-00A818977629}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="65">
   <si>
     <t>id</t>
   </si>
@@ -222,6 +222,18 @@
   </si>
   <si>
     <t>fijo_alternativo</t>
+  </si>
+  <si>
+    <t>rugby</t>
+  </si>
+  <si>
+    <t>Rugby 7</t>
+  </si>
+  <si>
+    <t>tiroarco</t>
+  </si>
+  <si>
+    <t>Tiro con arco</t>
   </si>
 </sst>
 </file>
@@ -593,7 +605,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{259D404A-F656-47E9-B6EB-214B2E007FEA}">
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1188,7 +1200,7 @@
         <v>13</v>
       </c>
       <c r="K17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L17" t="s">
         <v>59</v>
@@ -1262,6 +1274,76 @@
       </c>
       <c r="L19" t="s">
         <v>58</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>61</v>
+      </c>
+      <c r="C20" t="s">
+        <v>62</v>
+      </c>
+      <c r="D20" t="s">
+        <v>51</v>
+      </c>
+      <c r="E20">
+        <v>2</v>
+      </c>
+      <c r="F20">
+        <v>4</v>
+      </c>
+      <c r="G20">
+        <v>100</v>
+      </c>
+      <c r="H20" t="s">
+        <v>13</v>
+      </c>
+      <c r="I20" t="s">
+        <v>13</v>
+      </c>
+      <c r="K20">
+        <v>4</v>
+      </c>
+      <c r="L20" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>63</v>
+      </c>
+      <c r="C21" t="s">
+        <v>64</v>
+      </c>
+      <c r="D21" t="s">
+        <v>50</v>
+      </c>
+      <c r="E21">
+        <v>5</v>
+      </c>
+      <c r="F21">
+        <v>2</v>
+      </c>
+      <c r="G21">
+        <v>100</v>
+      </c>
+      <c r="H21" t="s">
+        <v>13</v>
+      </c>
+      <c r="I21" t="s">
+        <v>13</v>
+      </c>
+      <c r="K21">
+        <v>3</v>
+      </c>
+      <c r="L21" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>